<commit_message>
New yolo model ran with 15epochs and 30 patience. I also set the calibration to be per image, which means that the model will recalibrate for each image instead of using a single calibration for all images. This should improve the accuracy of the measurements, especially if there is variation in the distance between the camera and the straws in different images.
</commit_message>
<xml_diff>
--- a/straw_results.xlsx
+++ b/straw_results.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -39,10 +39,22 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
+      <color rgb="002E4057"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="15">
     <fill>
       <patternFill/>
     </fill>
@@ -57,6 +69,61 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00EAF4FB"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0000C8FF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00008CFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0000FF00"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="000050FF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFF00"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DCDC00"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FF00FF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="000080FF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0080FF00"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C8C8C8"/>
       </patternFill>
     </fill>
   </fills>
@@ -86,7 +153,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -100,7 +167,30 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -185,7 +275,7 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>1</row>
+      <row>14</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="3810000" cy="2857500"/>
@@ -196,6 +286,31 @@
       </nvPicPr>
       <blipFill>
         <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>15</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="3810000" cy="2857500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="2" name="Image 2" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId2"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -498,7 +613,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N11"/>
+  <dimension ref="A1:N14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -592,29 +707,31 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>IMG_2735.jpg</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="n">
+          <t>IMG_2730.jpg</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>0.1</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>17.932</v>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Straight</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="C2" s="2" t="n">
-        <v>145.032</v>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>Curved</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="b">
-        <v>0</v>
-      </c>
       <c r="F2" s="2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>RECONSTRUCTED</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -623,41 +740,39 @@
         </is>
       </c>
       <c r="I2" s="2" t="n">
-        <v>0.955</v>
-      </c>
-      <c r="J2" s="2" t="inlineStr">
-        <is>
-          <t>true_endpoint</t>
-        </is>
+        <v>0.949</v>
+      </c>
+      <c r="J2" s="2" t="n">
+        <v/>
       </c>
       <c r="K2" s="2" t="n">
-        <v>207</v>
+        <v>31</v>
       </c>
       <c r="L2" s="2" t="n">
-        <v>1.1467</v>
+        <v>1.0804</v>
       </c>
       <c r="M2" s="2" t="n">
-        <v>0.5911217723986145</v>
+        <v>0.5519991299409421</v>
       </c>
       <c r="N2" s="2" t="n">
-        <v>0.591122</v>
+        <v>0.551999</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>IMG_2735.jpg</t>
+          <t>IMG_2730.jpg</t>
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>214.358</v>
+        <v>115.31</v>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>Straight</t>
+          <t>Curved</t>
         </is>
       </c>
       <c r="E3" s="3" t="b">
@@ -677,7 +792,7 @@
         </is>
       </c>
       <c r="I3" s="3" t="n">
-        <v>0.9409999999999999</v>
+        <v>0.9389999999999999</v>
       </c>
       <c r="J3" s="3" t="inlineStr">
         <is>
@@ -685,37 +800,37 @@
         </is>
       </c>
       <c r="K3" s="3" t="n">
-        <v>287</v>
+        <v>178</v>
       </c>
       <c r="L3" s="3" t="n">
-        <v>1.082</v>
+        <v>1.1148</v>
       </c>
       <c r="M3" s="3" t="n">
-        <v>0.5911217723986145</v>
+        <v>0.5519991299409421</v>
       </c>
       <c r="N3" s="3" t="n">
-        <v>0.591122</v>
+        <v>0.551999</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>IMG_2735.jpg</t>
+          <t>IMG_2730.jpg</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>235.841</v>
+        <v>176.314</v>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Curved</t>
+          <t>Straight</t>
         </is>
       </c>
       <c r="E4" s="2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F4" s="2" t="b">
         <v>0</v>
@@ -731,7 +846,7 @@
         </is>
       </c>
       <c r="I4" s="2" t="n">
-        <v>0.9330000000000001</v>
+        <v>0.9</v>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
@@ -739,29 +854,31 @@
         </is>
       </c>
       <c r="K4" s="2" t="n">
-        <v>325</v>
+        <v>291</v>
       </c>
       <c r="L4" s="2" t="n">
-        <v>1.1435</v>
+        <v>1.0862</v>
       </c>
       <c r="M4" s="2" t="n">
-        <v>0.5911217723986145</v>
+        <v>0.5519991299409421</v>
       </c>
       <c r="N4" s="2" t="n">
-        <v>0.591122</v>
+        <v>0.551999</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>IMG_2735.jpg</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="n">
-        <v>4</v>
+          <t>IMG_2730.jpg</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>4.0</t>
+        </is>
       </c>
       <c r="C5" s="3" t="n">
-        <v>113.468</v>
+        <v>25.092</v>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
@@ -772,11 +889,11 @@
         <v>1</v>
       </c>
       <c r="F5" s="3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>RECONSTRUCTED</t>
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr">
@@ -785,39 +902,35 @@
         </is>
       </c>
       <c r="I5" s="3" t="n">
-        <v>0.913</v>
-      </c>
-      <c r="J5" s="3" t="inlineStr">
-        <is>
-          <t>true_endpoint</t>
-        </is>
+        <v>0.764</v>
+      </c>
+      <c r="J5" s="3" t="n">
+        <v/>
       </c>
       <c r="K5" s="3" t="n">
-        <v>171</v>
+        <v>39</v>
       </c>
       <c r="L5" s="3" t="n">
-        <v>1.1095</v>
+        <v>1.1407</v>
       </c>
       <c r="M5" s="3" t="n">
-        <v>0.5911217723986145</v>
+        <v>0.5519991299409421</v>
       </c>
       <c r="N5" s="3" t="n">
-        <v>0.591122</v>
+        <v>0.551999</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>IMG_2735.jpg</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>5.1</t>
-        </is>
+          <t>IMG_2740.jpg</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="n">
+        <v>3</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>30.476</v>
+        <v>152.506</v>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
@@ -825,14 +938,14 @@
         </is>
       </c>
       <c r="E6" s="2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F6" s="2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>RECONSTRUCTED</t>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
@@ -841,37 +954,37 @@
         </is>
       </c>
       <c r="I6" s="2" t="n">
-        <v>0.862</v>
-      </c>
-      <c r="J6" s="2" t="n">
-        <v/>
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>true_endpoint</t>
+        </is>
       </c>
       <c r="K6" s="2" t="n">
-        <v>48</v>
+        <v>223</v>
       </c>
       <c r="L6" s="2" t="n">
-        <v>1.085</v>
+        <v>1.098</v>
       </c>
       <c r="M6" s="2" t="n">
-        <v>0.5911217723986145</v>
+        <v>0.5708634448442826</v>
       </c>
       <c r="N6" s="2" t="n">
-        <v>0.591122</v>
+        <v>0.570863</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>IMG_2735.jpg</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>5.2</t>
-        </is>
+          <t>IMG_2740.jpg</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>4</v>
       </c>
       <c r="C7" s="3" t="n">
-        <v>16.002</v>
+        <v>142.483</v>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
@@ -879,14 +992,14 @@
         </is>
       </c>
       <c r="E7" s="3" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F7" s="3" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>RECONSTRUCTED</t>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="H7" s="3" t="inlineStr">
@@ -895,35 +1008,37 @@
         </is>
       </c>
       <c r="I7" s="3" t="n">
-        <v>0.862</v>
-      </c>
-      <c r="J7" s="3" t="n">
-        <v/>
+        <v>0.9389999999999999</v>
+      </c>
+      <c r="J7" s="3" t="inlineStr">
+        <is>
+          <t>true_endpoint</t>
+        </is>
       </c>
       <c r="K7" s="3" t="n">
-        <v>26</v>
+        <v>210</v>
       </c>
       <c r="L7" s="3" t="n">
-        <v>1.126</v>
+        <v>1.1396</v>
       </c>
       <c r="M7" s="3" t="n">
-        <v>0.5911217723986145</v>
+        <v>0.5708634448442826</v>
       </c>
       <c r="N7" s="3" t="n">
-        <v>0.591122</v>
+        <v>0.570863</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>IMG_2735.jpg</t>
+          <t>IMG_2740.jpg</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C8" s="2" t="n">
-        <v>159.827</v>
+        <v>113.812</v>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
@@ -931,7 +1046,7 @@
         </is>
       </c>
       <c r="E8" s="2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F8" s="2" t="b">
         <v>0</v>
@@ -947,7 +1062,7 @@
         </is>
       </c>
       <c r="I8" s="2" t="n">
-        <v>0.822</v>
+        <v>0.928</v>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
@@ -955,29 +1070,31 @@
         </is>
       </c>
       <c r="K8" s="2" t="n">
-        <v>237</v>
+        <v>178</v>
       </c>
       <c r="L8" s="2" t="n">
-        <v>1.1732</v>
+        <v>1.1235</v>
       </c>
       <c r="M8" s="2" t="n">
-        <v>0.5911217723986145</v>
+        <v>0.5708634448442826</v>
       </c>
       <c r="N8" s="2" t="n">
-        <v>0.591122</v>
+        <v>0.570863</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>IMG_2735.jpg</t>
-        </is>
-      </c>
-      <c r="B9" s="3" t="n">
-        <v>7</v>
+          <t>IMG_2740.jpg</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>6.0</t>
+        </is>
       </c>
       <c r="C9" s="3" t="n">
-        <v>235.092</v>
+        <v>12.836</v>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
@@ -985,14 +1102,14 @@
         </is>
       </c>
       <c r="E9" s="3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F9" s="3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>RECONSTRUCTED</t>
         </is>
       </c>
       <c r="H9" s="3" t="inlineStr">
@@ -1001,37 +1118,37 @@
         </is>
       </c>
       <c r="I9" s="3" t="n">
-        <v>0.791</v>
-      </c>
-      <c r="J9" s="3" t="inlineStr">
-        <is>
-          <t>true_endpoint</t>
-        </is>
+        <v>0.855</v>
+      </c>
+      <c r="J9" s="3" t="n">
+        <v/>
       </c>
       <c r="K9" s="3" t="n">
-        <v>349</v>
+        <v>21</v>
       </c>
       <c r="L9" s="3" t="n">
-        <v>1.1943</v>
+        <v>1.1415</v>
       </c>
       <c r="M9" s="3" t="n">
-        <v>0.5911217723986145</v>
+        <v>0.5708634448442826</v>
       </c>
       <c r="N9" s="3" t="n">
-        <v>0.591122</v>
+        <v>0.570863</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>IMG_2735.jpg</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="n">
-        <v>8</v>
+          <t>IMG_2740.jpg</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>6.1</t>
+        </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>96.29000000000001</v>
+        <v>38.704</v>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
@@ -1042,11 +1159,11 @@
         <v>1</v>
       </c>
       <c r="F10" s="2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>RECONSTRUCTED</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
@@ -1055,39 +1172,35 @@
         </is>
       </c>
       <c r="I10" s="2" t="n">
-        <v>0.761</v>
-      </c>
-      <c r="J10" s="2" t="inlineStr">
-        <is>
-          <t>true_endpoint</t>
-        </is>
+        <v>0.855</v>
+      </c>
+      <c r="J10" s="2" t="n">
+        <v/>
       </c>
       <c r="K10" s="2" t="n">
-        <v>132</v>
+        <v>63</v>
       </c>
       <c r="L10" s="2" t="n">
-        <v>1.0792</v>
+        <v>1.0913</v>
       </c>
       <c r="M10" s="2" t="n">
-        <v>0.5911217723986145</v>
+        <v>0.5708634448442826</v>
       </c>
       <c r="N10" s="2" t="n">
-        <v>0.591122</v>
+        <v>0.570863</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>IMG_2735.jpg</t>
-        </is>
-      </c>
-      <c r="B11" s="3" t="inlineStr">
-        <is>
-          <t>11.1</t>
-        </is>
+          <t>IMG_2740.jpg</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>7</v>
       </c>
       <c r="C11" s="3" t="n">
-        <v>38.304</v>
+        <v>245.733</v>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
@@ -1098,35 +1211,199 @@
         <v>1</v>
       </c>
       <c r="F11" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t>yolo</t>
+        </is>
+      </c>
+      <c r="I11" s="3" t="n">
+        <v>0.8100000000000001</v>
+      </c>
+      <c r="J11" s="3" t="inlineStr">
+        <is>
+          <t>true_endpoint</t>
+        </is>
+      </c>
+      <c r="K11" s="3" t="n">
+        <v>354</v>
+      </c>
+      <c r="L11" s="3" t="n">
+        <v>1.174</v>
+      </c>
+      <c r="M11" s="3" t="n">
+        <v>0.5708634448442826</v>
+      </c>
+      <c r="N11" s="3" t="n">
+        <v>0.570863</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>IMG_2740.jpg</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>8.1</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="n">
+        <v>33.999</v>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Curved</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="G11" s="3" t="inlineStr">
+      <c r="F12" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
         <is>
           <t>RECONSTRUCTED</t>
         </is>
       </c>
-      <c r="H11" s="3" t="inlineStr">
+      <c r="H12" s="2" t="inlineStr">
         <is>
           <t>yolo</t>
         </is>
       </c>
-      <c r="I11" s="3" t="n">
-        <v>0.551</v>
-      </c>
-      <c r="J11" s="3" t="n">
+      <c r="I12" s="2" t="n">
+        <v>0.6909999999999999</v>
+      </c>
+      <c r="J12" s="2" t="n">
         <v/>
       </c>
-      <c r="K11" s="3" t="n">
-        <v>60</v>
-      </c>
-      <c r="L11" s="3" t="n">
-        <v>1.5675</v>
-      </c>
-      <c r="M11" s="3" t="n">
-        <v>0.5911217723986145</v>
-      </c>
-      <c r="N11" s="3" t="n">
-        <v>0.591122</v>
+      <c r="K12" s="2" t="n">
+        <v>56</v>
+      </c>
+      <c r="L12" s="2" t="n">
+        <v>1.4006</v>
+      </c>
+      <c r="M12" s="2" t="n">
+        <v>0.5708634448442826</v>
+      </c>
+      <c r="N12" s="2" t="n">
+        <v>0.570863</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>IMG_2740.jpg</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>9.0</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="n">
+        <v>38.133</v>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>Straight</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="F13" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>RECONSTRUCTED</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>yolo</t>
+        </is>
+      </c>
+      <c r="I13" s="3" t="n">
+        <v>0.674</v>
+      </c>
+      <c r="J13" s="3" t="n">
+        <v/>
+      </c>
+      <c r="K13" s="3" t="n">
+        <v>62</v>
+      </c>
+      <c r="L13" s="3" t="n">
+        <v>1.0945</v>
+      </c>
+      <c r="M13" s="3" t="n">
+        <v>0.5708634448442826</v>
+      </c>
+      <c r="N13" s="3" t="n">
+        <v>0.570863</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>IMG_2740.jpg</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="C14" s="2" t="n">
+        <v>81.95099999999999</v>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Straight</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="F14" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>yolo</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="n">
+        <v>0.603</v>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>true_endpoint</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="n">
+        <v>140</v>
+      </c>
+      <c r="L14" s="2" t="n">
+        <v>1.0315</v>
+      </c>
+      <c r="M14" s="2" t="n">
+        <v>0.5708634448442826</v>
+      </c>
+      <c r="N14" s="2" t="n">
+        <v>0.570863</v>
       </c>
     </row>
   </sheetData>
@@ -1140,11 +1417,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
     <col width="100" customWidth="1" min="2" max="2"/>
+    <col width="6" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="52" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1158,16 +1438,192 @@
           <t>Overlay</t>
         </is>
       </c>
-    </row>
-    <row r="2" ht="225" customHeight="1">
-      <c r="A2" s="5" t="inlineStr">
-        <is>
-          <t>IMG_2735.jpg
-10 straw(s)</t>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>Color Key — Overlay Image Guide</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1">
+      <c r="C2" s="6" t="inlineStr">
+        <is>
+          <t>Color</t>
+        </is>
+      </c>
+      <c r="D2" s="6" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
+      <c r="E2" s="6" t="inlineStr">
+        <is>
+          <t>What it means</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="40" customHeight="1">
+      <c r="C3" s="7" t="inlineStr"/>
+      <c r="D3" s="8" t="inlineStr">
+        <is>
+          <t>Measured path (cyan)</t>
+        </is>
+      </c>
+      <c r="E3" s="9" t="inlineStr">
+        <is>
+          <t>The skeleton path traced through each straw from endpoint to endpoint. Length is calculated along this line.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="40" customHeight="1">
+      <c r="C4" s="10" t="inlineStr"/>
+      <c r="D4" s="8" t="inlineStr">
+        <is>
+          <t>Reconstructed path (orange-blue)</t>
+        </is>
+      </c>
+      <c r="E4" s="9" t="inlineStr">
+        <is>
+          <t>Path traced through a crossing/overlap region where two straws intersect. The algorithm separated them using angle matching.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="40" customHeight="1">
+      <c r="C5" s="11" t="inlineStr"/>
+      <c r="D5" s="8" t="inlineStr">
+        <is>
+          <t>Endpoints — normal (green)</t>
+        </is>
+      </c>
+      <c r="E5" s="9" t="inlineStr">
+        <is>
+          <t>The two tip points of a cleanly detected straw with no crossing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="40" customHeight="1">
+      <c r="C6" s="12" t="inlineStr"/>
+      <c r="D6" s="8" t="inlineStr">
+        <is>
+          <t>Endpoints — reconstructed (orange)</t>
+        </is>
+      </c>
+      <c r="E6" s="9" t="inlineStr">
+        <is>
+          <t>Tip points of a straw that was separated from a crossing. These mark where the reconstructed straw begins and ends.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="40" customHeight="1">
+      <c r="C7" s="13" t="inlineStr"/>
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>Branch points (cyan dots)</t>
+        </is>
+      </c>
+      <c r="E7" s="9" t="inlineStr">
+        <is>
+          <t>Points in the skeleton where 3 or more paths meet — indicates a crossing between two or more straws.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="40" customHeight="1">
+      <c r="C8" s="14" t="inlineStr"/>
+      <c r="D8" s="8" t="inlineStr">
+        <is>
+          <t>Endpoint markers (light cyan circles)</t>
+        </is>
+      </c>
+      <c r="E8" s="9" t="inlineStr">
+        <is>
+          <t>All raw skeleton endpoints detected before pairing — shown during overlap analysis to visualise candidate straw tips.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="40" customHeight="1">
+      <c r="C9" s="15" t="inlineStr"/>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>Crossing centroid (white cross)</t>
+        </is>
+      </c>
+      <c r="E9" s="9" t="inlineStr">
+        <is>
+          <t>The geometric center of all branch points in an overlap region. Used as the reference point for angle-based endpoint pairing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="40" customHeight="1">
+      <c r="C10" s="16" t="inlineStr"/>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>Pair line — set 1 (magenta)</t>
+        </is>
+      </c>
+      <c r="E10" s="9" t="inlineStr">
+        <is>
+          <t>Visual line connecting a matched endpoint pair (straw 1 through a crossing).</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="40" customHeight="1">
+      <c r="C11" s="17" t="inlineStr"/>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>Pair line — set 2 (orange)</t>
+        </is>
+      </c>
+      <c r="E11" s="9" t="inlineStr">
+        <is>
+          <t>Visual line connecting a matched endpoint pair (straw 2 through a crossing).</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="40" customHeight="1">
+      <c r="C12" s="18" t="inlineStr"/>
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>Pair line — set 3 (green)</t>
+        </is>
+      </c>
+      <c r="E12" s="9" t="inlineStr">
+        <is>
+          <t>Visual line connecting a matched endpoint pair (straw 3 through a crossing).</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="40" customHeight="1">
+      <c r="C13" s="19" t="inlineStr"/>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>Status bar (bottom of image)</t>
+        </is>
+      </c>
+      <c r="E13" s="9" t="inlineStr">
+        <is>
+          <t>Shows detection mode, number of straws measured, mask count, and the calibration ratio used (mm per pixel).</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="225" customHeight="1">
+      <c r="A15" s="20" t="inlineStr">
+        <is>
+          <t>IMG_2730.jpg
+4 straw(s)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="225" customHeight="1">
+      <c r="A16" s="20" t="inlineStr">
+        <is>
+          <t>IMG_2740.jpg
+9 straw(s)</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="C1:E1"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Test 100 was to fine tune the relationship between the confidence threshold and the resulting measurements. I found that 0.5 was a good balance for the YOLO model, giving accurate measurements without too many false positives. This should help improve the overall performance of the system when deployed in real-world conditions.Merged_Final is the best version of my code
</commit_message>
<xml_diff>
--- a/straw_results.xlsx
+++ b/straw_results.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -39,22 +39,10 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="002E4057"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="15">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -69,61 +57,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00EAF4FB"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="0000C8FF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00008CFF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="0000FF00"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="000050FF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFFF00"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00DCDC00"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFFFFF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FF00FF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="000080FF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="0080FF00"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00C8C8C8"/>
       </patternFill>
     </fill>
   </fills>
@@ -153,7 +86,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -167,30 +100,7 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -275,7 +185,7 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>14</row>
+      <row>1</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="3810000" cy="2857500"/>
@@ -286,31 +196,6 @@
       </nvPicPr>
       <blipFill>
         <a:blip cstate="print" r:embed="rId1"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>1</col>
-      <colOff>0</colOff>
-      <row>15</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="3810000" cy="2857500"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="2" name="Image 2" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId2"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -613,7 +498,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N14"/>
+  <dimension ref="A1:N10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -707,16 +592,14 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>IMG_2730.jpg</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>0.1</t>
-        </is>
+          <t>IMG_2733.jpg</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>17.932</v>
+        <v>342.225</v>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
@@ -724,14 +607,14 @@
         </is>
       </c>
       <c r="E2" s="2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F2" s="2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>RECONSTRUCTED</t>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -740,43 +623,45 @@
         </is>
       </c>
       <c r="I2" s="2" t="n">
-        <v>0.949</v>
-      </c>
-      <c r="J2" s="2" t="n">
+        <v>0.896</v>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>bfs</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="n">
+        <v>540</v>
+      </c>
+      <c r="L2" s="2" t="n">
         <v/>
       </c>
-      <c r="K2" s="2" t="n">
-        <v>31</v>
-      </c>
-      <c r="L2" s="2" t="n">
-        <v>1.0804</v>
-      </c>
       <c r="M2" s="2" t="n">
-        <v>0.5519991299409421</v>
+        <v>0.5579540406553007</v>
       </c>
       <c r="N2" s="2" t="n">
-        <v>0.551999</v>
+        <v>0.5579539999999999</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>IMG_2730.jpg</t>
+          <t>IMG_2733.jpg</t>
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>115.31</v>
+        <v>106.534</v>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>Curved</t>
+          <t>Straight</t>
         </is>
       </c>
       <c r="E3" s="3" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F3" s="3" t="b">
         <v>0</v>
@@ -792,37 +677,37 @@
         </is>
       </c>
       <c r="I3" s="3" t="n">
-        <v>0.9389999999999999</v>
+        <v>0.896</v>
       </c>
       <c r="J3" s="3" t="inlineStr">
         <is>
-          <t>true_endpoint</t>
+          <t>bfs</t>
         </is>
       </c>
       <c r="K3" s="3" t="n">
-        <v>178</v>
+        <v>153</v>
       </c>
       <c r="L3" s="3" t="n">
-        <v>1.1148</v>
+        <v/>
       </c>
       <c r="M3" s="3" t="n">
-        <v>0.5519991299409421</v>
+        <v>0.5579540406553007</v>
       </c>
       <c r="N3" s="3" t="n">
-        <v>0.551999</v>
+        <v>0.5579539999999999</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>IMG_2730.jpg</t>
+          <t>IMG_2733.jpg</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>176.314</v>
+        <v>42.755</v>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
@@ -830,7 +715,7 @@
         </is>
       </c>
       <c r="E4" s="2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F4" s="2" t="b">
         <v>0</v>
@@ -846,54 +731,52 @@
         </is>
       </c>
       <c r="I4" s="2" t="n">
-        <v>0.9</v>
+        <v>0.892</v>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>true_endpoint</t>
+          <t>bfs</t>
         </is>
       </c>
       <c r="K4" s="2" t="n">
-        <v>291</v>
+        <v>71</v>
       </c>
       <c r="L4" s="2" t="n">
-        <v>1.0862</v>
+        <v/>
       </c>
       <c r="M4" s="2" t="n">
-        <v>0.5519991299409421</v>
+        <v>0.5579540406553007</v>
       </c>
       <c r="N4" s="2" t="n">
-        <v>0.551999</v>
+        <v>0.5579539999999999</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>IMG_2730.jpg</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>4.0</t>
-        </is>
+          <t>IMG_2733.jpg</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>4</v>
       </c>
       <c r="C5" s="3" t="n">
-        <v>25.092</v>
+        <v>248.704</v>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>Curved</t>
+          <t>Straight</t>
         </is>
       </c>
       <c r="E5" s="3" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F5" s="3" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>RECONSTRUCTED</t>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr">
@@ -902,35 +785,37 @@
         </is>
       </c>
       <c r="I5" s="3" t="n">
-        <v>0.764</v>
-      </c>
-      <c r="J5" s="3" t="n">
+        <v>0.891</v>
+      </c>
+      <c r="J5" s="3" t="inlineStr">
+        <is>
+          <t>bfs</t>
+        </is>
+      </c>
+      <c r="K5" s="3" t="n">
+        <v>414</v>
+      </c>
+      <c r="L5" s="3" t="n">
         <v/>
       </c>
-      <c r="K5" s="3" t="n">
-        <v>39</v>
-      </c>
-      <c r="L5" s="3" t="n">
-        <v>1.1407</v>
-      </c>
       <c r="M5" s="3" t="n">
-        <v>0.5519991299409421</v>
+        <v>0.5579540406553007</v>
       </c>
       <c r="N5" s="3" t="n">
-        <v>0.551999</v>
+        <v>0.5579539999999999</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>IMG_2740.jpg</t>
+          <t>IMG_2733.jpg</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>152.506</v>
+        <v>190.874</v>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
@@ -954,41 +839,41 @@
         </is>
       </c>
       <c r="I6" s="2" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.866</v>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>true_endpoint</t>
+          <t>bfs</t>
         </is>
       </c>
       <c r="K6" s="2" t="n">
-        <v>223</v>
+        <v>465</v>
       </c>
       <c r="L6" s="2" t="n">
-        <v>1.098</v>
+        <v/>
       </c>
       <c r="M6" s="2" t="n">
-        <v>0.5708634448442826</v>
+        <v>0.5579540406553007</v>
       </c>
       <c r="N6" s="2" t="n">
-        <v>0.570863</v>
+        <v>0.5579539999999999</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>IMG_2740.jpg</t>
+          <t>IMG_2733.jpg</t>
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C7" s="3" t="n">
-        <v>142.483</v>
+        <v>120.42</v>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>Curved</t>
+          <t>Straight</t>
         </is>
       </c>
       <c r="E7" s="3" t="b">
@@ -1008,37 +893,39 @@
         </is>
       </c>
       <c r="I7" s="3" t="n">
-        <v>0.9389999999999999</v>
+        <v>0.853</v>
       </c>
       <c r="J7" s="3" t="inlineStr">
         <is>
-          <t>true_endpoint</t>
+          <t>bfs</t>
         </is>
       </c>
       <c r="K7" s="3" t="n">
-        <v>210</v>
+        <v>266</v>
       </c>
       <c r="L7" s="3" t="n">
-        <v>1.1396</v>
+        <v/>
       </c>
       <c r="M7" s="3" t="n">
-        <v>0.5708634448442826</v>
+        <v>0.5579540406553007</v>
       </c>
       <c r="N7" s="3" t="n">
-        <v>0.570863</v>
+        <v>0.5579539999999999</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>IMG_2740.jpg</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="n">
-        <v>5</v>
+          <t>IMG_2733.jpg</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>7.0</t>
+        </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>113.812</v>
+        <v>15.893</v>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
@@ -1049,11 +936,11 @@
         <v>1</v>
       </c>
       <c r="F8" s="2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>RECONSTRUCTED</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
@@ -1062,39 +949,37 @@
         </is>
       </c>
       <c r="I8" s="2" t="n">
-        <v>0.928</v>
-      </c>
-      <c r="J8" s="2" t="inlineStr">
-        <is>
-          <t>true_endpoint</t>
-        </is>
+        <v>0.773</v>
+      </c>
+      <c r="J8" s="2" t="n">
+        <v/>
       </c>
       <c r="K8" s="2" t="n">
-        <v>178</v>
+        <v>27</v>
       </c>
       <c r="L8" s="2" t="n">
-        <v>1.1235</v>
+        <v>1.1533</v>
       </c>
       <c r="M8" s="2" t="n">
-        <v>0.5708634448442826</v>
+        <v>0.5579540406553007</v>
       </c>
       <c r="N8" s="2" t="n">
-        <v>0.570863</v>
+        <v>0.5579539999999999</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>IMG_2740.jpg</t>
+          <t>IMG_2733.jpg</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>6.0</t>
+          <t>7.1</t>
         </is>
       </c>
       <c r="C9" s="3" t="n">
-        <v>12.836</v>
+        <v>11.334</v>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
@@ -1118,41 +1003,41 @@
         </is>
       </c>
       <c r="I9" s="3" t="n">
-        <v>0.855</v>
+        <v>0.773</v>
       </c>
       <c r="J9" s="3" t="n">
         <v/>
       </c>
       <c r="K9" s="3" t="n">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="L9" s="3" t="n">
-        <v>1.1415</v>
+        <v>1.4935</v>
       </c>
       <c r="M9" s="3" t="n">
-        <v>0.5708634448442826</v>
+        <v>0.5579540406553007</v>
       </c>
       <c r="N9" s="3" t="n">
-        <v>0.570863</v>
+        <v>0.5579539999999999</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>IMG_2740.jpg</t>
+          <t>IMG_2733.jpg</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>6.1</t>
+          <t>8.0</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>38.704</v>
+        <v>10.776</v>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Straight</t>
+          <t>Curved</t>
         </is>
       </c>
       <c r="E10" s="2" t="b">
@@ -1172,238 +1057,22 @@
         </is>
       </c>
       <c r="I10" s="2" t="n">
-        <v>0.855</v>
+        <v>0.716</v>
       </c>
       <c r="J10" s="2" t="n">
         <v/>
       </c>
       <c r="K10" s="2" t="n">
-        <v>63</v>
+        <v>17</v>
       </c>
       <c r="L10" s="2" t="n">
-        <v>1.0913</v>
+        <v>1.1041</v>
       </c>
       <c r="M10" s="2" t="n">
-        <v>0.5708634448442826</v>
+        <v>0.5579540406553007</v>
       </c>
       <c r="N10" s="2" t="n">
-        <v>0.570863</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>IMG_2740.jpg</t>
-        </is>
-      </c>
-      <c r="B11" s="3" t="n">
-        <v>7</v>
-      </c>
-      <c r="C11" s="3" t="n">
-        <v>245.733</v>
-      </c>
-      <c r="D11" s="3" t="inlineStr">
-        <is>
-          <t>Curved</t>
-        </is>
-      </c>
-      <c r="E11" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="F11" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="G11" s="3" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="H11" s="3" t="inlineStr">
-        <is>
-          <t>yolo</t>
-        </is>
-      </c>
-      <c r="I11" s="3" t="n">
-        <v>0.8100000000000001</v>
-      </c>
-      <c r="J11" s="3" t="inlineStr">
-        <is>
-          <t>true_endpoint</t>
-        </is>
-      </c>
-      <c r="K11" s="3" t="n">
-        <v>354</v>
-      </c>
-      <c r="L11" s="3" t="n">
-        <v>1.174</v>
-      </c>
-      <c r="M11" s="3" t="n">
-        <v>0.5708634448442826</v>
-      </c>
-      <c r="N11" s="3" t="n">
-        <v>0.570863</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>IMG_2740.jpg</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>8.1</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="n">
-        <v>33.999</v>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>Curved</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="F12" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="G12" s="2" t="inlineStr">
-        <is>
-          <t>RECONSTRUCTED</t>
-        </is>
-      </c>
-      <c r="H12" s="2" t="inlineStr">
-        <is>
-          <t>yolo</t>
-        </is>
-      </c>
-      <c r="I12" s="2" t="n">
-        <v>0.6909999999999999</v>
-      </c>
-      <c r="J12" s="2" t="n">
-        <v/>
-      </c>
-      <c r="K12" s="2" t="n">
-        <v>56</v>
-      </c>
-      <c r="L12" s="2" t="n">
-        <v>1.4006</v>
-      </c>
-      <c r="M12" s="2" t="n">
-        <v>0.5708634448442826</v>
-      </c>
-      <c r="N12" s="2" t="n">
-        <v>0.570863</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>IMG_2740.jpg</t>
-        </is>
-      </c>
-      <c r="B13" s="3" t="inlineStr">
-        <is>
-          <t>9.0</t>
-        </is>
-      </c>
-      <c r="C13" s="3" t="n">
-        <v>38.133</v>
-      </c>
-      <c r="D13" s="3" t="inlineStr">
-        <is>
-          <t>Straight</t>
-        </is>
-      </c>
-      <c r="E13" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="F13" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="G13" s="3" t="inlineStr">
-        <is>
-          <t>RECONSTRUCTED</t>
-        </is>
-      </c>
-      <c r="H13" s="3" t="inlineStr">
-        <is>
-          <t>yolo</t>
-        </is>
-      </c>
-      <c r="I13" s="3" t="n">
-        <v>0.674</v>
-      </c>
-      <c r="J13" s="3" t="n">
-        <v/>
-      </c>
-      <c r="K13" s="3" t="n">
-        <v>62</v>
-      </c>
-      <c r="L13" s="3" t="n">
-        <v>1.0945</v>
-      </c>
-      <c r="M13" s="3" t="n">
-        <v>0.5708634448442826</v>
-      </c>
-      <c r="N13" s="3" t="n">
-        <v>0.570863</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>IMG_2740.jpg</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="C14" s="2" t="n">
-        <v>81.95099999999999</v>
-      </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>Straight</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="F14" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="G14" s="2" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-      <c r="H14" s="2" t="inlineStr">
-        <is>
-          <t>yolo</t>
-        </is>
-      </c>
-      <c r="I14" s="2" t="n">
-        <v>0.603</v>
-      </c>
-      <c r="J14" s="2" t="inlineStr">
-        <is>
-          <t>true_endpoint</t>
-        </is>
-      </c>
-      <c r="K14" s="2" t="n">
-        <v>140</v>
-      </c>
-      <c r="L14" s="2" t="n">
-        <v>1.0315</v>
-      </c>
-      <c r="M14" s="2" t="n">
-        <v>0.5708634448442826</v>
-      </c>
-      <c r="N14" s="2" t="n">
-        <v>0.570863</v>
+        <v>0.5579539999999999</v>
       </c>
     </row>
   </sheetData>
@@ -1417,14 +1086,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:B2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
     <col width="100" customWidth="1" min="2" max="2"/>
-    <col width="6" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
-    <col width="52" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1438,192 +1104,16 @@
           <t>Overlay</t>
         </is>
       </c>
-      <c r="C1" s="5" t="inlineStr">
-        <is>
-          <t>Color Key — Overlay Image Guide</t>
-        </is>
-      </c>
     </row>
-    <row r="2" ht="18" customHeight="1">
-      <c r="C2" s="6" t="inlineStr">
-        <is>
-          <t>Color</t>
-        </is>
-      </c>
-      <c r="D2" s="6" t="inlineStr">
-        <is>
-          <t>Element</t>
-        </is>
-      </c>
-      <c r="E2" s="6" t="inlineStr">
-        <is>
-          <t>What it means</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="40" customHeight="1">
-      <c r="C3" s="7" t="inlineStr"/>
-      <c r="D3" s="8" t="inlineStr">
-        <is>
-          <t>Measured path (cyan)</t>
-        </is>
-      </c>
-      <c r="E3" s="9" t="inlineStr">
-        <is>
-          <t>The skeleton path traced through each straw from endpoint to endpoint. Length is calculated along this line.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="40" customHeight="1">
-      <c r="C4" s="10" t="inlineStr"/>
-      <c r="D4" s="8" t="inlineStr">
-        <is>
-          <t>Reconstructed path (orange-blue)</t>
-        </is>
-      </c>
-      <c r="E4" s="9" t="inlineStr">
-        <is>
-          <t>Path traced through a crossing/overlap region where two straws intersect. The algorithm separated them using angle matching.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="40" customHeight="1">
-      <c r="C5" s="11" t="inlineStr"/>
-      <c r="D5" s="8" t="inlineStr">
-        <is>
-          <t>Endpoints — normal (green)</t>
-        </is>
-      </c>
-      <c r="E5" s="9" t="inlineStr">
-        <is>
-          <t>The two tip points of a cleanly detected straw with no crossing.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="40" customHeight="1">
-      <c r="C6" s="12" t="inlineStr"/>
-      <c r="D6" s="8" t="inlineStr">
-        <is>
-          <t>Endpoints — reconstructed (orange)</t>
-        </is>
-      </c>
-      <c r="E6" s="9" t="inlineStr">
-        <is>
-          <t>Tip points of a straw that was separated from a crossing. These mark where the reconstructed straw begins and ends.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="40" customHeight="1">
-      <c r="C7" s="13" t="inlineStr"/>
-      <c r="D7" s="8" t="inlineStr">
-        <is>
-          <t>Branch points (cyan dots)</t>
-        </is>
-      </c>
-      <c r="E7" s="9" t="inlineStr">
-        <is>
-          <t>Points in the skeleton where 3 or more paths meet — indicates a crossing between two or more straws.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="40" customHeight="1">
-      <c r="C8" s="14" t="inlineStr"/>
-      <c r="D8" s="8" t="inlineStr">
-        <is>
-          <t>Endpoint markers (light cyan circles)</t>
-        </is>
-      </c>
-      <c r="E8" s="9" t="inlineStr">
-        <is>
-          <t>All raw skeleton endpoints detected before pairing — shown during overlap analysis to visualise candidate straw tips.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="40" customHeight="1">
-      <c r="C9" s="15" t="inlineStr"/>
-      <c r="D9" s="8" t="inlineStr">
-        <is>
-          <t>Crossing centroid (white cross)</t>
-        </is>
-      </c>
-      <c r="E9" s="9" t="inlineStr">
-        <is>
-          <t>The geometric center of all branch points in an overlap region. Used as the reference point for angle-based endpoint pairing.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="40" customHeight="1">
-      <c r="C10" s="16" t="inlineStr"/>
-      <c r="D10" s="8" t="inlineStr">
-        <is>
-          <t>Pair line — set 1 (magenta)</t>
-        </is>
-      </c>
-      <c r="E10" s="9" t="inlineStr">
-        <is>
-          <t>Visual line connecting a matched endpoint pair (straw 1 through a crossing).</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="40" customHeight="1">
-      <c r="C11" s="17" t="inlineStr"/>
-      <c r="D11" s="8" t="inlineStr">
-        <is>
-          <t>Pair line — set 2 (orange)</t>
-        </is>
-      </c>
-      <c r="E11" s="9" t="inlineStr">
-        <is>
-          <t>Visual line connecting a matched endpoint pair (straw 2 through a crossing).</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="40" customHeight="1">
-      <c r="C12" s="18" t="inlineStr"/>
-      <c r="D12" s="8" t="inlineStr">
-        <is>
-          <t>Pair line — set 3 (green)</t>
-        </is>
-      </c>
-      <c r="E12" s="9" t="inlineStr">
-        <is>
-          <t>Visual line connecting a matched endpoint pair (straw 3 through a crossing).</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="40" customHeight="1">
-      <c r="C13" s="19" t="inlineStr"/>
-      <c r="D13" s="8" t="inlineStr">
-        <is>
-          <t>Status bar (bottom of image)</t>
-        </is>
-      </c>
-      <c r="E13" s="9" t="inlineStr">
-        <is>
-          <t>Shows detection mode, number of straws measured, mask count, and the calibration ratio used (mm per pixel).</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="225" customHeight="1">
-      <c r="A15" s="20" t="inlineStr">
-        <is>
-          <t>IMG_2730.jpg
-4 straw(s)</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="225" customHeight="1">
-      <c r="A16" s="20" t="inlineStr">
-        <is>
-          <t>IMG_2740.jpg
+    <row r="2" ht="225" customHeight="1">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>IMG_2733.jpg
 9 straw(s)</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="C1:E1"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>

</xml_diff>